<commit_message>
48. Key Excel Functions: SUM, SUMIF, SUMIFS
</commit_message>
<xml_diff>
--- a/The Complete Financial Analyst Course/Section 5/48. Key Excel Functions SUM, SUMIF, SUMIFS/39.+Sum-Sumif-Sumifs-Exercise+-Unsolved.xlsx
+++ b/The Complete Financial Analyst Course/Section 5/48. Key Excel Functions SUM, SUMIF, SUMIFS/39.+Sum-Sumif-Sumifs-Exercise+-Unsolved.xlsx
@@ -1,19 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="17030"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28025"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C091FA91-D45B-41A5-B477-8667400E99CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="28680" yWindow="270" windowWidth="29040" windowHeight="17640" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exercise" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -346,7 +358,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -499,10 +511,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -519,13 +529,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -537,11 +541,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -856,8 +869,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:J20"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="B2:H20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.42578125" customWidth="1"/>
@@ -869,1856 +882,1844 @@
     <col min="8" max="8" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="12" t="s">
+    <row r="2" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-    </row>
-    <row r="3" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-    </row>
-    <row r="4" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="13"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="1"/>
-    </row>
-    <row r="5" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="14">
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+    </row>
+    <row r="3" spans="2:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="15"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
+    </row>
+    <row r="4" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+    </row>
+    <row r="5" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="10">
         <v>1</v>
       </c>
-      <c r="C5" s="16"/>
-      <c r="D5" s="17" t="s">
+      <c r="C5" s="12"/>
+      <c r="D5" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
-      <c r="I5" s="1"/>
-    </row>
-    <row r="6" spans="1:10" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="15"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
-      <c r="I6" s="1"/>
-    </row>
-    <row r="7" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="1"/>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="1"/>
-    </row>
-    <row r="8" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="13"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="13"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="13"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-    </row>
-    <row r="9" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="14">
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="13"/>
+    </row>
+    <row r="6" spans="2:8" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="11"/>
+      <c r="C6" s="12"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="13"/>
+    </row>
+    <row r="7" spans="2:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
+    </row>
+    <row r="8" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
+    </row>
+    <row r="9" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="10">
         <v>2</v>
       </c>
-      <c r="C9" s="16"/>
-      <c r="D9" s="17" t="s">
+      <c r="C9" s="12"/>
+      <c r="D9" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="17"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-    </row>
-    <row r="10" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="15"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
-    </row>
-    <row r="11" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B11" s="11"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
-    </row>
-    <row r="12" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="13"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="2"/>
-      <c r="J12" s="2"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B13" s="14">
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13"/>
+      <c r="H9" s="13"/>
+    </row>
+    <row r="10" spans="2:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="11"/>
+      <c r="C10" s="12"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="13"/>
+    </row>
+    <row r="11" spans="2:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B11" s="14"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="14"/>
+      <c r="H11" s="14"/>
+    </row>
+    <row r="12" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B13" s="10">
         <v>3</v>
       </c>
-      <c r="C13" s="16"/>
-      <c r="D13" s="17" t="s">
+      <c r="C13" s="12"/>
+      <c r="D13" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="17"/>
-      <c r="H13" s="17"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
-    </row>
-    <row r="14" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="15"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="17"/>
-      <c r="I14" s="2"/>
-      <c r="J14" s="2"/>
-    </row>
-    <row r="15" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B15" s="11"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="11"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
-    </row>
-    <row r="16" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="13"/>
+    </row>
+    <row r="14" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="11"/>
+      <c r="C14" s="12"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="13"/>
+      <c r="H14" s="13"/>
+    </row>
+    <row r="15" spans="2:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B15" s="14"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="14"/>
+      <c r="F15" s="14"/>
+      <c r="G15" s="14"/>
+      <c r="H15" s="14"/>
+    </row>
+    <row r="16" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="19" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="D13:H14"/>
-    <mergeCell ref="B15:H15"/>
-    <mergeCell ref="B8:H8"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:H10"/>
-    <mergeCell ref="B11:H11"/>
     <mergeCell ref="B7:H7"/>
     <mergeCell ref="B2:H3"/>
     <mergeCell ref="B4:H4"/>
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="C5:C6"/>
     <mergeCell ref="D5:H6"/>
+    <mergeCell ref="B8:H8"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:H10"/>
+    <mergeCell ref="B11:H11"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="D13:H14"/>
+    <mergeCell ref="B15:H15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:M51"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.85546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.7109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.28515625" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.85546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="23" style="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.42578125" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="9.140625" style="6"/>
+    <col min="1" max="1" width="9.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23" style="4" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="4">
         <v>12.2</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="6">
+      <c r="G2" s="4">
         <v>111</v>
       </c>
-      <c r="H2" s="6">
+      <c r="H2" s="4">
         <v>95.66</v>
       </c>
-      <c r="I2" s="6">
+      <c r="I2" s="4">
         <v>77.48</v>
       </c>
-      <c r="J2" s="6">
+      <c r="J2" s="4">
         <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="4">
         <v>12.1</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="6">
+      <c r="G3" s="4">
         <v>115</v>
       </c>
-      <c r="H3" s="6">
+      <c r="H3" s="4">
         <v>145.30000000000001</v>
       </c>
-      <c r="I3" s="6">
+      <c r="I3" s="4">
         <v>117.69</v>
       </c>
-      <c r="J3" s="6">
+      <c r="J3" s="4">
         <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="4">
         <v>14.1</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G4" s="6">
+      <c r="G4" s="4">
         <v>108</v>
       </c>
-      <c r="H4" s="6">
+      <c r="H4" s="4">
         <v>159.83000000000001</v>
       </c>
-      <c r="I4" s="6">
+      <c r="I4" s="4">
         <v>124.67</v>
       </c>
-      <c r="J4" s="6">
+      <c r="J4" s="4">
         <v>37</v>
       </c>
-      <c r="K4" s="18" t="s">
+      <c r="K4" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="L4" s="18"/>
-      <c r="M4" s="8"/>
+      <c r="L4" s="16"/>
+      <c r="M4" s="6">
+        <f>SUM(J2:J51)</f>
+        <v>2246</v>
+      </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="4">
         <v>14</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="G5" s="6">
+      <c r="G5" s="4">
         <v>106</v>
       </c>
-      <c r="H5" s="6">
+      <c r="H5" s="4">
         <v>76.37</v>
       </c>
-      <c r="I5" s="6">
+      <c r="I5" s="4">
         <v>66.44</v>
       </c>
-      <c r="J5" s="6">
+      <c r="J5" s="4">
         <v>53</v>
       </c>
-      <c r="K5" s="18" t="s">
+      <c r="K5" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="L5" s="18"/>
-      <c r="M5" s="10"/>
+      <c r="L5" s="17"/>
+      <c r="M5" s="8">
+        <f>SUMIF(A2:A51,"Sony",J2:J51)</f>
+        <v>191</v>
+      </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="4">
         <v>12.1</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="G6" s="6">
+      <c r="G6" s="4">
         <v>367</v>
       </c>
-      <c r="H6" s="6">
+      <c r="H6" s="4">
         <v>254.26</v>
       </c>
-      <c r="I6" s="6">
+      <c r="I6" s="4">
         <v>221.21</v>
       </c>
-      <c r="J6" s="6">
+      <c r="J6" s="4">
         <v>52</v>
       </c>
-      <c r="K6" s="18" t="s">
+      <c r="K6" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="L6" s="18"/>
-      <c r="M6" s="9"/>
+      <c r="L6" s="16"/>
+      <c r="M6" s="7">
+        <f>SUMIFS(J2:J51, A2:A51,"Sony",B2:B51,"Japan")</f>
+        <v>137</v>
+      </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="4">
         <v>10</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="G7" s="6">
+      <c r="G7" s="4">
         <v>168</v>
       </c>
-      <c r="H7" s="6">
+      <c r="H7" s="4">
         <v>121.1</v>
       </c>
-      <c r="I7" s="6">
+      <c r="I7" s="4">
         <v>94.46</v>
       </c>
-      <c r="J7" s="6">
+      <c r="J7" s="4">
         <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="4">
         <v>14.1</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G8" s="6">
+      <c r="G8" s="4">
         <v>137</v>
       </c>
-      <c r="H8" s="6">
+      <c r="H8" s="4">
         <v>240.53</v>
       </c>
-      <c r="I8" s="6">
+      <c r="I8" s="4">
         <v>214.07</v>
       </c>
-      <c r="J8" s="6">
+      <c r="J8" s="4">
         <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="4">
         <v>12.1</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G9" s="6">
+      <c r="G9" s="4">
         <v>126</v>
       </c>
-      <c r="H9" s="6">
+      <c r="H9" s="4">
         <v>138.01</v>
       </c>
-      <c r="I9" s="6">
+      <c r="I9" s="4">
         <v>107.65</v>
       </c>
-      <c r="J9" s="6">
+      <c r="J9" s="4">
         <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="4">
         <v>12.2</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G10" s="6">
+      <c r="G10" s="4">
         <v>130</v>
       </c>
-      <c r="H10" s="6">
+      <c r="H10" s="4">
         <v>227.75</v>
       </c>
-      <c r="I10" s="6">
+      <c r="I10" s="4">
         <v>179.92</v>
       </c>
-      <c r="J10" s="6">
+      <c r="J10" s="4">
         <v>54</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="4">
         <v>12</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="G11" s="6">
+      <c r="G11" s="4">
         <v>195</v>
       </c>
-      <c r="H11" s="6">
+      <c r="H11" s="4">
         <v>203.4</v>
       </c>
-      <c r="I11" s="6">
+      <c r="I11" s="4">
         <v>142.38</v>
       </c>
-      <c r="J11" s="6">
+      <c r="J11" s="4">
         <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="4">
         <v>12.1</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="G12" s="6">
+      <c r="G12" s="4">
         <v>115</v>
       </c>
-      <c r="H12" s="6">
+      <c r="H12" s="4">
         <v>87.21</v>
       </c>
-      <c r="I12" s="6">
+      <c r="I12" s="4">
         <v>75.87</v>
       </c>
-      <c r="J12" s="6">
+      <c r="J12" s="4">
         <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="4">
         <v>12</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="F13" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="G13" s="6">
+      <c r="G13" s="4">
         <v>341</v>
       </c>
-      <c r="H13" s="6">
+      <c r="H13" s="4">
         <v>168.28</v>
       </c>
-      <c r="I13" s="6">
+      <c r="I13" s="4">
         <v>121.16</v>
       </c>
-      <c r="J13" s="6">
+      <c r="J13" s="4">
         <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="D14" s="6">
+      <c r="D14" s="4">
         <v>12.2</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="G14" s="6">
+      <c r="G14" s="4">
         <v>113</v>
       </c>
-      <c r="H14" s="6">
+      <c r="H14" s="4">
         <v>73.27</v>
       </c>
-      <c r="I14" s="6">
+      <c r="I14" s="4">
         <v>63.74</v>
       </c>
-      <c r="J14" s="6">
+      <c r="J14" s="4">
         <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D15" s="6">
+      <c r="D15" s="4">
         <v>14.1</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="E15" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="G15" s="6">
+      <c r="G15" s="4">
         <v>124</v>
       </c>
-      <c r="H15" s="6">
+      <c r="H15" s="4">
         <v>107.15</v>
       </c>
-      <c r="I15" s="6">
+      <c r="I15" s="4">
         <v>76.08</v>
       </c>
-      <c r="J15" s="6">
+      <c r="J15" s="4">
         <v>51</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
+      <c r="A16" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="D16" s="6">
+      <c r="D16" s="4">
         <v>14</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E16" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="F16" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="G16" s="6">
+      <c r="G16" s="4">
         <v>116</v>
       </c>
-      <c r="H16" s="6">
+      <c r="H16" s="4">
         <v>157.59</v>
       </c>
-      <c r="I16" s="6">
+      <c r="I16" s="4">
         <v>138.68</v>
       </c>
-      <c r="J16" s="6">
+      <c r="J16" s="4">
         <v>43</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="D17" s="6">
+      <c r="D17" s="4">
         <v>10</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="E17" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="F17" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G17" s="6">
+      <c r="G17" s="4">
         <v>105</v>
       </c>
-      <c r="H17" s="6">
+      <c r="H17" s="4">
         <v>108.96</v>
       </c>
-      <c r="I17" s="6">
+      <c r="I17" s="4">
         <v>91.53</v>
       </c>
-      <c r="J17" s="6">
+      <c r="J17" s="4">
         <v>37</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D18" s="6">
+      <c r="D18" s="4">
         <v>12.1</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="E18" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="F18" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="G18" s="6">
+      <c r="G18" s="4">
         <v>136</v>
       </c>
-      <c r="H18" s="6">
+      <c r="H18" s="4">
         <v>147.33000000000001</v>
       </c>
-      <c r="I18" s="6">
+      <c r="I18" s="4">
         <v>116.39</v>
       </c>
-      <c r="J18" s="6">
+      <c r="J18" s="4">
         <v>61</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="D19" s="6">
+      <c r="D19" s="4">
         <v>9.1</v>
       </c>
-      <c r="E19" s="7" t="s">
+      <c r="E19" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F19" s="7" t="s">
+      <c r="F19" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="G19" s="6">
+      <c r="G19" s="4">
         <v>453</v>
       </c>
-      <c r="H19" s="6">
+      <c r="H19" s="4">
         <v>305.27</v>
       </c>
-      <c r="I19" s="6">
+      <c r="I19" s="4">
         <v>225.9</v>
       </c>
-      <c r="J19" s="6">
+      <c r="J19" s="4">
         <v>46</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A20" s="6" t="s">
+      <c r="A20" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="D20" s="6">
+      <c r="D20" s="4">
         <v>12.2</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="E20" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="F20" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G20" s="6">
+      <c r="G20" s="4">
         <v>195</v>
       </c>
-      <c r="H20" s="6">
+      <c r="H20" s="4">
         <v>84.75</v>
       </c>
-      <c r="I20" s="6">
+      <c r="I20" s="4">
         <v>60.17</v>
       </c>
-      <c r="J20" s="6">
+      <c r="J20" s="4">
         <v>42</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A21" s="6" t="s">
+      <c r="A21" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="D21" s="6">
+      <c r="D21" s="4">
         <v>10.1</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="E21" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F21" s="7" t="s">
+      <c r="F21" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="G21" s="6">
+      <c r="G21" s="4">
         <v>260</v>
       </c>
-      <c r="H21" s="6">
+      <c r="H21" s="4">
         <v>168.42</v>
       </c>
-      <c r="I21" s="6">
+      <c r="I21" s="4">
         <v>151.58000000000001</v>
       </c>
-      <c r="J21" s="6">
+      <c r="J21" s="4">
         <v>27</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" s="6" t="s">
+      <c r="A22" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D22" s="6">
+      <c r="D22" s="4">
         <v>12.1</v>
       </c>
-      <c r="E22" s="7" t="s">
+      <c r="E22" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F22" s="7" t="s">
+      <c r="F22" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="G22" s="6">
+      <c r="G22" s="4">
         <v>140</v>
       </c>
-      <c r="H22" s="6">
+      <c r="H22" s="4">
         <v>268.5</v>
       </c>
-      <c r="I22" s="6">
+      <c r="I22" s="4">
         <v>222.86</v>
       </c>
-      <c r="J22" s="6">
+      <c r="J22" s="4">
         <v>54</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A23" s="6" t="s">
+      <c r="A23" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D23" s="6">
+      <c r="D23" s="4">
         <v>14.2</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="E23" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="F23" s="7" t="s">
+      <c r="F23" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G23" s="6">
+      <c r="G23" s="4">
         <v>147</v>
       </c>
-      <c r="H23" s="6">
+      <c r="H23" s="4">
         <v>176.88</v>
       </c>
-      <c r="I23" s="6">
+      <c r="I23" s="4">
         <v>132.66</v>
       </c>
-      <c r="J23" s="6">
+      <c r="J23" s="4">
         <v>39</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A24" s="6" t="s">
+      <c r="A24" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C24" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D24" s="6">
+      <c r="D24" s="4">
         <v>10</v>
       </c>
-      <c r="E24" s="7" t="s">
+      <c r="E24" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F24" s="7" t="s">
+      <c r="F24" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="G24" s="6">
+      <c r="G24" s="4">
         <v>150</v>
       </c>
-      <c r="H24" s="6">
+      <c r="H24" s="4">
         <v>259.18</v>
       </c>
-      <c r="I24" s="6">
+      <c r="I24" s="4">
         <v>220.3</v>
       </c>
-      <c r="J24" s="6">
+      <c r="J24" s="4">
         <v>64</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A25" s="6" t="s">
+      <c r="A25" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="C25" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="D25" s="6">
+      <c r="D25" s="4">
         <v>12</v>
       </c>
-      <c r="E25" s="7" t="s">
+      <c r="E25" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F25" s="7" t="s">
+      <c r="F25" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G25" s="6">
+      <c r="G25" s="4">
         <v>150</v>
       </c>
-      <c r="H25" s="6">
+      <c r="H25" s="4">
         <v>149.57</v>
       </c>
-      <c r="I25" s="6">
+      <c r="I25" s="4">
         <v>121.15</v>
       </c>
-      <c r="J25" s="6">
+      <c r="J25" s="4">
         <v>56</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A26" s="6" t="s">
+      <c r="A26" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="C26" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="D26" s="6">
+      <c r="D26" s="4">
         <v>10</v>
       </c>
-      <c r="E26" s="7" t="s">
+      <c r="E26" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F26" s="7" t="s">
+      <c r="F26" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="G26" s="6">
+      <c r="G26" s="4">
         <v>120</v>
       </c>
-      <c r="H26" s="6">
+      <c r="H26" s="4">
         <v>101.73</v>
       </c>
-      <c r="I26" s="6">
+      <c r="I26" s="4">
         <v>90.54</v>
       </c>
-      <c r="J26" s="6">
+      <c r="J26" s="4">
         <v>54</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A27" s="6" t="s">
+      <c r="A27" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="D27" s="6">
+      <c r="D27" s="4">
         <v>12.1</v>
       </c>
-      <c r="E27" s="7" t="s">
+      <c r="E27" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F27" s="7" t="s">
+      <c r="F27" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="G27" s="6">
+      <c r="G27" s="4">
         <v>131</v>
       </c>
-      <c r="H27" s="6">
+      <c r="H27" s="4">
         <v>150.29</v>
       </c>
-      <c r="I27" s="6">
+      <c r="I27" s="4">
         <v>117.23</v>
       </c>
-      <c r="J27" s="6">
+      <c r="J27" s="4">
         <v>61</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A28" s="6" t="s">
+      <c r="A28" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="C28" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="D28" s="6">
+      <c r="D28" s="4">
         <v>12.2</v>
       </c>
-      <c r="E28" s="7" t="s">
+      <c r="E28" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F28" s="7" t="s">
+      <c r="F28" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="G28" s="6">
+      <c r="G28" s="4">
         <v>124</v>
       </c>
-      <c r="H28" s="6">
+      <c r="H28" s="4">
         <v>69.150000000000006</v>
       </c>
-      <c r="I28" s="6">
+      <c r="I28" s="4">
         <v>62.24</v>
       </c>
-      <c r="J28" s="6">
+      <c r="J28" s="4">
         <v>42</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A29" s="6" t="s">
+      <c r="A29" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="D29" s="6">
+      <c r="D29" s="4">
         <v>12.2</v>
       </c>
-      <c r="E29" s="7" t="s">
+      <c r="E29" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="F29" s="7" t="s">
+      <c r="F29" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="G29" s="6">
+      <c r="G29" s="4">
         <v>214</v>
       </c>
-      <c r="H29" s="6">
+      <c r="H29" s="4">
         <v>250.79</v>
       </c>
-      <c r="I29" s="6">
+      <c r="I29" s="4">
         <v>198.12</v>
       </c>
-      <c r="J29" s="6">
+      <c r="J29" s="4">
         <v>52</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C30" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="D30" s="6">
+      <c r="D30" s="4">
         <v>12.1</v>
       </c>
-      <c r="E30" s="7" t="s">
+      <c r="E30" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F30" s="7" t="s">
+      <c r="F30" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G30" s="6">
+      <c r="G30" s="4">
         <v>153</v>
       </c>
-      <c r="H30" s="6">
+      <c r="H30" s="4">
         <v>102.89</v>
       </c>
-      <c r="I30" s="6">
+      <c r="I30" s="4">
         <v>88.49</v>
       </c>
-      <c r="J30" s="6">
+      <c r="J30" s="4">
         <v>50</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A31" s="6" t="s">
+      <c r="A31" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="C31" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="D31" s="6">
+      <c r="D31" s="4">
         <v>10.1</v>
       </c>
-      <c r="E31" s="7" t="s">
+      <c r="E31" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F31" s="7" t="s">
+      <c r="F31" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="G31" s="6">
+      <c r="G31" s="4">
         <v>120</v>
       </c>
-      <c r="H31" s="6">
+      <c r="H31" s="4">
         <v>365.75</v>
       </c>
-      <c r="I31" s="6">
+      <c r="I31" s="4">
         <v>274.31</v>
       </c>
-      <c r="J31" s="6">
+      <c r="J31" s="4">
         <v>50</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A32" s="6" t="s">
+      <c r="A32" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C32" s="6" t="s">
+      <c r="C32" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="D32" s="6">
+      <c r="D32" s="4">
         <v>12.2</v>
       </c>
-      <c r="E32" s="7" t="s">
+      <c r="E32" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F32" s="7" t="s">
+      <c r="F32" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="G32" s="6">
+      <c r="G32" s="4">
         <v>113</v>
       </c>
-      <c r="H32" s="6">
+      <c r="H32" s="4">
         <v>73.27</v>
       </c>
-      <c r="I32" s="6">
+      <c r="I32" s="4">
         <v>65.94</v>
       </c>
-      <c r="J32" s="6">
+      <c r="J32" s="4">
         <v>71</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A33" s="6" t="s">
+      <c r="A33" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="B33" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C33" s="6" t="s">
+      <c r="C33" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="D33" s="6">
+      <c r="D33" s="4">
         <v>9.2899999999999991</v>
       </c>
-      <c r="E33" s="7" t="s">
+      <c r="E33" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F33" s="7" t="s">
+      <c r="F33" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="G33" s="6">
+      <c r="G33" s="4">
         <v>185</v>
       </c>
-      <c r="H33" s="6">
+      <c r="H33" s="4">
         <v>192.63</v>
       </c>
-      <c r="I33" s="6">
+      <c r="I33" s="4">
         <v>154.1</v>
       </c>
-      <c r="J33" s="6">
+      <c r="J33" s="4">
         <v>51</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A34" s="6" t="s">
+      <c r="A34" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="B34" s="6" t="s">
+      <c r="B34" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C34" s="6" t="s">
+      <c r="C34" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="D34" s="6">
+      <c r="D34" s="4">
         <v>12</v>
       </c>
-      <c r="E34" s="7" t="s">
+      <c r="E34" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F34" s="7" t="s">
+      <c r="F34" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="G34" s="6">
+      <c r="G34" s="4">
         <v>183</v>
       </c>
-      <c r="H34" s="6">
+      <c r="H34" s="4">
         <v>77.53</v>
       </c>
-      <c r="I34" s="6">
+      <c r="I34" s="4">
         <v>59.7</v>
       </c>
-      <c r="J34" s="6">
+      <c r="J34" s="4">
         <v>43</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A35" s="6" t="s">
+      <c r="A35" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="B35" s="6" t="s">
+      <c r="B35" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C35" s="6" t="s">
+      <c r="C35" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="D35" s="6">
+      <c r="D35" s="4">
         <v>14.2</v>
       </c>
-      <c r="E35" s="7" t="s">
+      <c r="E35" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F35" s="7" t="s">
+      <c r="F35" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="G35" s="6">
+      <c r="G35" s="4">
         <v>156</v>
       </c>
-      <c r="H35" s="6">
+      <c r="H35" s="4">
         <v>249.86</v>
       </c>
-      <c r="I35" s="6">
+      <c r="I35" s="4">
         <v>182.4</v>
       </c>
-      <c r="J35" s="6">
+      <c r="J35" s="4">
         <v>15</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A36" s="6" t="s">
+      <c r="A36" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="B36" s="6" t="s">
+      <c r="B36" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C36" s="6" t="s">
+      <c r="C36" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="D36" s="6">
+      <c r="D36" s="4">
         <v>12</v>
       </c>
-      <c r="E36" s="7" t="s">
+      <c r="E36" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F36" s="7" t="s">
+      <c r="F36" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G36" s="6">
+      <c r="G36" s="4">
         <v>360</v>
       </c>
-      <c r="H36" s="6">
+      <c r="H36" s="4">
         <v>98.77</v>
       </c>
-      <c r="I36" s="6">
+      <c r="I36" s="4">
         <v>75.069999999999993</v>
       </c>
-      <c r="J36" s="6">
+      <c r="J36" s="4">
         <v>69</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A37" s="6" t="s">
+      <c r="A37" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="B37" s="6" t="s">
+      <c r="B37" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C37" s="6" t="s">
+      <c r="C37" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="D37" s="6">
+      <c r="D37" s="4">
         <v>14</v>
       </c>
-      <c r="E37" s="7" t="s">
+      <c r="E37" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F37" s="7" t="s">
+      <c r="F37" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="G37" s="6">
+      <c r="G37" s="4">
         <v>171</v>
       </c>
-      <c r="H37" s="6">
+      <c r="H37" s="4">
         <v>266.39999999999998</v>
       </c>
-      <c r="I37" s="6">
+      <c r="I37" s="4">
         <v>229.1</v>
       </c>
-      <c r="J37" s="6">
+      <c r="J37" s="4">
         <v>37</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A38" s="6" t="s">
+      <c r="A38" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="B38" s="6" t="s">
+      <c r="B38" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C38" s="6" t="s">
+      <c r="C38" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="D38" s="6">
+      <c r="D38" s="4">
         <v>14.1</v>
       </c>
-      <c r="E38" s="7" t="s">
+      <c r="E38" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F38" s="7" t="s">
+      <c r="F38" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G38" s="6">
+      <c r="G38" s="4">
         <v>155</v>
       </c>
-      <c r="H38" s="6">
+      <c r="H38" s="4">
         <v>268.5</v>
       </c>
-      <c r="I38" s="6">
+      <c r="I38" s="4">
         <v>196.01</v>
       </c>
-      <c r="J38" s="6">
+      <c r="J38" s="4">
         <v>53</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A39" s="6" t="s">
+      <c r="A39" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B39" s="6" t="s">
+      <c r="B39" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C39" s="6" t="s">
+      <c r="C39" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="D39" s="6">
+      <c r="D39" s="4">
         <v>12.1</v>
       </c>
-      <c r="E39" s="7" t="s">
+      <c r="E39" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F39" s="7" t="s">
+      <c r="F39" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="G39" s="6">
+      <c r="G39" s="4">
         <v>336</v>
       </c>
-      <c r="H39" s="6">
+      <c r="H39" s="4">
         <v>523.19000000000005</v>
       </c>
-      <c r="I39" s="6">
+      <c r="I39" s="4">
         <v>413.32</v>
       </c>
-      <c r="J39" s="6">
+      <c r="J39" s="4">
         <v>52</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A40" s="6" t="s">
+      <c r="A40" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B40" s="6" t="s">
+      <c r="B40" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C40" s="6" t="s">
+      <c r="C40" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="D40" s="6">
+      <c r="D40" s="4">
         <v>10</v>
       </c>
-      <c r="E40" s="7" t="s">
+      <c r="E40" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F40" s="7" t="s">
+      <c r="F40" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="G40" s="6">
+      <c r="G40" s="4">
         <v>167</v>
       </c>
-      <c r="H40" s="6">
+      <c r="H40" s="4">
         <v>271.32</v>
       </c>
-      <c r="I40" s="6">
+      <c r="I40" s="4">
         <v>211.63</v>
       </c>
-      <c r="J40" s="6">
+      <c r="J40" s="4">
         <v>66</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A41" s="6" t="s">
+      <c r="A41" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B41" s="6" t="s">
+      <c r="B41" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C41" s="6" t="s">
+      <c r="C41" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D41" s="6">
+      <c r="D41" s="4">
         <v>14.1</v>
       </c>
-      <c r="E41" s="7" t="s">
+      <c r="E41" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F41" s="7" t="s">
+      <c r="F41" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="G41" s="6">
+      <c r="G41" s="4">
         <v>124</v>
       </c>
-      <c r="H41" s="6">
+      <c r="H41" s="4">
         <v>107.15</v>
       </c>
-      <c r="I41" s="6">
+      <c r="I41" s="4">
         <v>81.430000000000007</v>
       </c>
-      <c r="J41" s="6">
+      <c r="J41" s="4">
         <v>32</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A42" s="6" t="s">
+      <c r="A42" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B42" s="6" t="s">
+      <c r="B42" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C42" s="6" t="s">
+      <c r="C42" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D42" s="6">
+      <c r="D42" s="4">
         <v>10</v>
       </c>
-      <c r="E42" s="7" t="s">
+      <c r="E42" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F42" s="7" t="s">
+      <c r="F42" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="G42" s="6">
+      <c r="G42" s="4">
         <v>180</v>
       </c>
-      <c r="H42" s="6">
+      <c r="H42" s="4">
         <v>132.01</v>
       </c>
-      <c r="I42" s="6">
+      <c r="I42" s="4">
         <v>116.17</v>
       </c>
-      <c r="J42" s="6">
+      <c r="J42" s="4">
         <v>37</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A43" s="6" t="s">
+      <c r="A43" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B43" s="6" t="s">
+      <c r="B43" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C43" s="6" t="s">
+      <c r="C43" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="D43" s="6">
+      <c r="D43" s="4">
         <v>14.1</v>
       </c>
-      <c r="E43" s="7" t="s">
+      <c r="E43" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F43" s="7" t="s">
+      <c r="F43" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="G43" s="6">
+      <c r="G43" s="4">
         <v>170</v>
       </c>
-      <c r="H43" s="6">
+      <c r="H43" s="4">
         <v>169.65</v>
       </c>
-      <c r="I43" s="6">
+      <c r="I43" s="4">
         <v>144.19999999999999</v>
       </c>
-      <c r="J43" s="6">
+      <c r="J43" s="4">
         <v>54</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A44" s="6" t="s">
+      <c r="A44" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B44" s="6" t="s">
+      <c r="B44" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C44" s="6" t="s">
+      <c r="C44" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="D44" s="6">
+      <c r="D44" s="4">
         <v>12</v>
       </c>
-      <c r="E44" s="7" t="s">
+      <c r="E44" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F44" s="7" t="s">
+      <c r="F44" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="G44" s="6">
+      <c r="G44" s="4">
         <v>183</v>
       </c>
-      <c r="H44" s="6">
+      <c r="H44" s="4">
         <v>147.69</v>
       </c>
-      <c r="I44" s="6">
+      <c r="I44" s="4">
         <v>104.86</v>
       </c>
-      <c r="J44" s="6">
+      <c r="J44" s="4">
         <v>44</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A45" s="6" t="s">
+      <c r="A45" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B45" s="6" t="s">
+      <c r="B45" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C45" s="6" t="s">
+      <c r="C45" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="D45" s="6">
+      <c r="D45" s="4">
         <v>12.2</v>
       </c>
-      <c r="E45" s="7" t="s">
+      <c r="E45" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F45" s="7" t="s">
+      <c r="F45" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="G45" s="6">
+      <c r="G45" s="4">
         <v>106</v>
       </c>
-      <c r="H45" s="6">
+      <c r="H45" s="4">
         <v>70.88</v>
       </c>
-      <c r="I45" s="6">
+      <c r="I45" s="4">
         <v>57.41</v>
       </c>
-      <c r="J45" s="6">
+      <c r="J45" s="4">
         <v>17</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A46" s="6" t="s">
+      <c r="A46" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B46" s="6" t="s">
+      <c r="B46" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C46" s="6" t="s">
+      <c r="C46" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="D46" s="6">
+      <c r="D46" s="4">
         <v>12.1</v>
       </c>
-      <c r="E46" s="7" t="s">
+      <c r="E46" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F46" s="7" t="s">
+      <c r="F46" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="G46" s="6">
+      <c r="G46" s="4">
         <v>140</v>
       </c>
-      <c r="H46" s="6">
+      <c r="H46" s="4">
         <v>111.49</v>
       </c>
-      <c r="I46" s="6">
+      <c r="I46" s="4">
         <v>88.08</v>
       </c>
-      <c r="J46" s="6">
+      <c r="J46" s="4">
         <v>17</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A47" s="6" t="s">
+      <c r="A47" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B47" s="6" t="s">
+      <c r="B47" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C47" s="6" t="s">
+      <c r="C47" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="D47" s="6">
+      <c r="D47" s="4">
         <v>12.1</v>
       </c>
-      <c r="E47" s="7" t="s">
+      <c r="E47" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F47" s="7" t="s">
+      <c r="F47" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G47" s="6">
+      <c r="G47" s="4">
         <v>132</v>
       </c>
-      <c r="H47" s="6">
+      <c r="H47" s="4">
         <v>84.75</v>
       </c>
-      <c r="I47" s="6">
+      <c r="I47" s="4">
         <v>68.650000000000006</v>
       </c>
-      <c r="J47" s="6">
+      <c r="J47" s="4">
         <v>37</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A48" s="6" t="s">
+      <c r="A48" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="B48" s="6" t="s">
+      <c r="B48" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C48" s="6" t="s">
+      <c r="C48" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="D48" s="6">
+      <c r="D48" s="4">
         <v>10.3</v>
       </c>
-      <c r="E48" s="7" t="s">
+      <c r="E48" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F48" s="7" t="s">
+      <c r="F48" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="G48" s="6">
+      <c r="G48" s="4">
         <v>481</v>
       </c>
-      <c r="H48" s="6">
+      <c r="H48" s="4">
         <v>370.3</v>
       </c>
-      <c r="I48" s="6">
+      <c r="I48" s="4">
         <v>274.02</v>
       </c>
-      <c r="J48" s="6">
+      <c r="J48" s="4">
         <v>51</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A49" s="6" t="s">
+      <c r="A49" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B49" s="6" t="s">
+      <c r="B49" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C49" s="6" t="s">
+      <c r="C49" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="D49" s="6">
+      <c r="D49" s="4">
         <v>12.1</v>
       </c>
-      <c r="E49" s="7" t="s">
+      <c r="E49" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F49" s="7" t="s">
+      <c r="F49" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="G49" s="6">
+      <c r="G49" s="4">
         <v>125</v>
       </c>
-      <c r="H49" s="6">
+      <c r="H49" s="4">
         <v>71.39</v>
       </c>
-      <c r="I49" s="6">
+      <c r="I49" s="4">
         <v>62.82</v>
       </c>
-      <c r="J49" s="6">
+      <c r="J49" s="4">
         <v>43</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A50" s="6" t="s">
+      <c r="A50" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B50" s="6" t="s">
+      <c r="B50" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C50" s="6" t="s">
+      <c r="C50" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D50" s="6">
+      <c r="D50" s="4">
         <v>12</v>
       </c>
-      <c r="E50" s="7" t="s">
+      <c r="E50" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F50" s="7" t="s">
+      <c r="F50" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="G50" s="6">
+      <c r="G50" s="4">
         <v>195</v>
       </c>
-      <c r="H50" s="6">
+      <c r="H50" s="4">
         <v>203.4</v>
       </c>
-      <c r="I50" s="6">
+      <c r="I50" s="4">
         <v>183.06</v>
       </c>
-      <c r="J50" s="6">
+      <c r="J50" s="4">
         <v>37</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A51" s="6" t="s">
+      <c r="A51" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B51" s="6" t="s">
+      <c r="B51" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C51" s="6" t="s">
+      <c r="C51" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="D51" s="6">
+      <c r="D51" s="4">
         <v>6</v>
       </c>
-      <c r="E51" s="7" t="s">
+      <c r="E51" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="F51" s="7" t="s">
+      <c r="F51" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="G51" s="6">
+      <c r="G51" s="4">
         <v>130</v>
       </c>
-      <c r="H51" s="6">
+      <c r="H51" s="4">
         <v>77.53</v>
       </c>
-      <c r="I51" s="6">
+      <c r="I51" s="4">
         <v>56.6</v>
       </c>
-      <c r="J51" s="6">
+      <c r="J51" s="4">
         <v>61</v>
       </c>
     </row>

</xml_diff>